<commit_message>
Synchronise les données avec les moteurs Livraison et Avant-vente
Met à jour les exports hebdomadaires avec le schéma harmonisé utilisé
par les moteurs Livraison et Avant-vente, et synchronise le calendrier
des événements RH.

Corrige le mismatch entre le code déployé et les données historiques
sans modifier les règles métier ni les moteurs.
</commit_message>
<xml_diff>
--- a/data_calendrier/calendrier_evenements.xlsx
+++ b/data_calendrier/calendrier_evenements.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="EVENEMENTS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="EVENEMENTS_RH" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -48,9 +50,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,6 +419,449 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>date_debut</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>date_fin</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>nom_evenement</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>nature</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>canal_diffusion</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>reduction_pct</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>45915</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>45930</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Lancement édition limitée «Cocon d'Hiver»</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Produit</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Lancement</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Réseaux sociaux</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Senteur limitée annonçant la saison automne-hiver</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>45981</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>45991</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Black Friday</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Campagne</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>TV + Réseaux sociaux</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>25</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Plus gros pic de vente de l'année</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>45992</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46015</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Noël</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Fête</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>TV + Email</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>15</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Packs cadeaux mis en avant, forte demande avant-vente</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>46027</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>46042</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Promo senteurs d'hiver</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Campagne</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>20</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Écoulement du stock post-fêtes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>46060</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>46067</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>St Valentin</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Fête</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Réseaux sociaux</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Pack duo mis en avant</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>46062</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>46067</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Lancement recharge « Étreinte — édition limitée »</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Produit</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Lancement</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Réseaux sociaux (social ads)</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>10</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Forte hausse avant-vente attendue, pas de crise SAV à ce stade — premiers retours d'intensité olfactive concentrés à partir de mars. Chevauche la campagne St Valentin (événement séparé).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>46073</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>46082</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Fête des Grands-Mères</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Fête</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Fête des Grands-Mères (1er dimanche de mars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>46137</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Lancement nouvelle couleur «Sable»</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Produit</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Lancement</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Réseaux sociaux</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Nouvelle teinte du diffuseur, demandes de personnalisation attendues</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>46173</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Fête des Mères</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Fête</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>TV + Réseaux sociaux</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>15</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Fête des Mères (dernier dimanche de mai)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Soldes d'été</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Campagne</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>10</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Campagne discrète, période plus calme</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Anniversaire Emyria (5 ans)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Campagne</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Réseaux sociaux + Email</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>10</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Campagne de fidélisation, pas de gros pic attendu</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -442,318 +888,347 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>canal_diffusion</t>
+          <t>nature</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>reduction_pct</t>
+          <t>perimetre</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>notes</t>
+          <t>description</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>45915</v>
       </c>
-      <c r="B2" s="1" t="n">
-        <v>45930</v>
+      <c r="B2" s="2" t="n">
+        <v>45915</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Lancement édition limitée «Cocon d'Hiver»</t>
+          <t>Arrivée Sofia (alternance)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Lancement produit</t>
+          <t>Staffing</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Réseaux sociaux</t>
+          <t>Arrivée</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Sofia</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Senteur limitée annonçant la saison automne-hiver</t>
+          <t>Début de l'alternance de Sofia.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>45981</v>
-      </c>
-      <c r="B3" s="1" t="n">
-        <v>45991</v>
+      <c r="A3" s="2" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46170</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Black Friday</t>
+          <t>Absence école Sofia (examen)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Campagne marketing</t>
+          <t>Staffing</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>TV + Réseaux sociaux</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>25</v>
+          <t>Absence</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Sofia</t>
+        </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Plus gros pic de vente de l'année</t>
+          <t>Journée d'examen — présence de la semaine ramenée à mercredi + vendredi (14h au lieu de 21h).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Sofia à temps plein (été, hors période scolaire)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Staffing</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Disponibilité élargie</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Sofia</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Pas de cours en juillet-août : présence entreprise à temps plein (lundi-vendredi, 35h/semaine) au lieu du rythme standard — décision narrative explicite, pas une semaine isolée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Fin d'alternance Sofia</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Staffing</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Départ</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Sofia</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Fin de l'alternance de Sofia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>46027</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>46027</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Arrivée Lucie (stage)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Staffing</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Arrivée</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Lucie</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Début du stage de Lucie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Fin de stage Lucie</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Staffing</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Départ</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Lucie</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Fin du stage de Lucie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
         <v>45992</v>
       </c>
-      <c r="B4" s="1" t="n">
-        <v>46015</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Noël</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Fête standard</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>TV + Email</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Packs cadeaux mis en avant, forte demande avant-vente</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>46027</v>
-      </c>
-      <c r="B5" s="1" t="n">
-        <v>46042</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Promo senteurs d'hiver</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Campagne marketing</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>20</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Écoulement du stock post-fêtes</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>46060</v>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>46067</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>St Valentin</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Fête standard</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Réseaux sociaux</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>10</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Pack duo mis en avant</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>46073</v>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>46082</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Fête des Grands-Mères</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Fête standard</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Fête des Grands-Mères (1er dimanche de mars)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>46122</v>
-      </c>
-      <c r="B8" s="1" t="n">
-        <v>46137</v>
+      <c r="B8" s="2" t="n">
+        <v>46022</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Lancement nouvelle couleur «Sable»</t>
+          <t>Renfort saisonnier Sam</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Lancement produit</t>
+          <t>Staffing</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Réseaux sociaux</t>
+          <t>Renfort</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Sam</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Nouvelle teinte du diffuseur, demandes de personnalisation attendues</t>
+          <t>Renfort pour le pic de Noël, périmètre avant-vente/livraison/après-vente simple (hors SAV produit). Temps plein (lundi-vendredi, 35h) sur la semaine observée du 15-21 décembre.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>46162</v>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>46173</v>
+      <c r="A9" s="2" t="n">
+        <v>46090</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>46096</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Fête des Mères</t>
+          <t>Absence Amine (congés)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Fête standard</t>
+          <t>Staffing</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>TV + Réseaux sociaux</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>15</v>
+          <t>Absence</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Amine</t>
+        </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Fête des Mères (dernier dimanche de mai)</t>
+          <t>Congés — semaine observée du 9-15 mars.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>46193</v>
-      </c>
-      <c r="B10" s="1" t="n">
-        <v>46203</v>
+      <c r="A10" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>46215</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Soldes d'été</t>
+          <t>Absence Amine (congés)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Campagne marketing</t>
+          <t>Staffing</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>10</v>
+          <t>Absence</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Amine</t>
+        </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Campagne discrète, période plus calme</t>
+          <t>Congés — semaine observée du 6-12 juillet 2026.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>46266</v>
-      </c>
-      <c r="B11" s="1" t="n">
-        <v>46280</v>
+      <c r="A11" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>46250</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Anniversaire Emyria (5 ans)</t>
+          <t>Absence Kristelle (congés)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Campagne marketing</t>
+          <t>Staffing</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Réseaux sociaux + Email</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>10</v>
+          <t>Absence</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Kristelle</t>
+        </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Campagne de fidélisation, pas de gros pic attendu</t>
+          <t>Congés — semaine observée du 10-16 août 2026.</t>
         </is>
       </c>
     </row>

</xml_diff>